<commit_message>
generating html file on assumptions log
</commit_message>
<xml_diff>
--- a/Assumptions_and_decisions/assumptions_and_decision_log_template.xlsx
+++ b/Assumptions_and_decisions/assumptions_and_decision_log_template.xlsx
@@ -4,14 +4,14 @@
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25601"/>
   <fileSharing readOnlyRecommended="1"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCA2BDE0-8E93-4A5C-9116-D7F0B384C674}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2C5AA40-ABE3-43B4-BB69-1110F510431D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Introduction" sheetId="11" r:id="rId1"/>
     <sheet name="Decisions &amp; Issues Register" sheetId="7" r:id="rId2"/>
-    <sheet name="Assumptions log " sheetId="6" r:id="rId3"/>
+    <sheet name="assumptions" sheetId="6" r:id="rId3"/>
     <sheet name="Quality &amp; Sensitivity Guide" sheetId="5" r:id="rId4"/>
     <sheet name="Risk Scoring Guide" sheetId="8" r:id="rId5"/>
     <sheet name="Ethics Log" sheetId="13" r:id="rId6"/>
@@ -39,35 +39,8 @@
 </workbook>
 </file>
 
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author>tc={A40347E3-87F8-48F5-90A0-735595EC1AE9}</author>
-    <author>tc={FF24A55A-270A-4BF5-9774-591A378EC420}</author>
-  </authors>
-  <commentList>
-    <comment ref="B4" authorId="0" shapeId="0" xr:uid="{A40347E3-87F8-48F5-90A0-735595EC1AE9}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    Provide a link to the methodology document.</t>
-      </text>
-    </comment>
-    <comment ref="J8" authorId="1" shapeId="0" xr:uid="{FF24A55A-270A-4BF5-9774-591A378EC420}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    There should also be a plain English description of what might be the likely impact on model output if the assumption is found to be false later in the analysis.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="76">
   <si>
     <t>This template aims to aid model production by providing a structured template for documentation</t>
   </si>
@@ -157,9 +130,6 @@
   </si>
   <si>
     <t>Reviewed by</t>
-  </si>
-  <si>
-    <t>Assumptions log for [Insert Model Name &amp; Financial Year of Interest]</t>
   </si>
   <si>
     <t>Assumption ID</t>
@@ -525,7 +495,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="24">
+  <borders count="21">
     <border>
       <left/>
       <right/>
@@ -606,17 +576,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -637,30 +596,10 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
       <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
       <top/>
       <bottom/>
       <diagonal/>
@@ -792,7 +731,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -870,28 +809,28 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="17" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -902,19 +841,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -923,16 +862,16 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="20" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -945,30 +884,18 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -978,7 +905,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1330,17 +1257,6 @@
 </a:theme>
 </file>
 
-<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
-<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="B4" dT="2022-06-28T10:22:12.43" personId="{00000000-0000-0000-0000-000000000000}" id="{A40347E3-87F8-48F5-90A0-735595EC1AE9}">
-    <text>Provide a link to the methodology document.</text>
-  </threadedComment>
-  <threadedComment ref="J8" dT="2022-06-28T09:56:47.28" personId="{00000000-0000-0000-0000-000000000000}" id="{FF24A55A-270A-4BF5-9774-591A378EC420}">
-    <text>There should also be a plain English description of what might be the likely impact on model output if the assumption is found to be false later in the analysis.</text>
-  </threadedComment>
-</ThreadedComments>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE0E718D-ABA6-478B-BFB8-19647D312746}">
   <dimension ref="B2:D18"/>
@@ -1804,12 +1720,12 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
-    <tabColor rgb="FF92D050"/>
+    <tabColor theme="0"/>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
-  <dimension ref="A2:S36"/>
+  <dimension ref="A1:S27"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.81640625" style="1" customWidth="1"/>
@@ -1831,256 +1747,267 @@
     <col min="20" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:19" s="9" customFormat="1" ht="23.5" x14ac:dyDescent="0.55000000000000004">
-      <c r="D2" s="10" t="s">
+    <row r="1" spans="1:19" ht="39" x14ac:dyDescent="0.35">
+      <c r="B1" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="I2" s="27" t="s">
-        <v>19</v>
-      </c>
-      <c r="K2" s="16"/>
-      <c r="L2" s="16"/>
-      <c r="M2" s="16"/>
-      <c r="N2" s="16"/>
-      <c r="O2" s="16"/>
-      <c r="P2" s="16"/>
-    </row>
-    <row r="3" spans="1:19" s="9" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="K3" s="16"/>
-      <c r="L3" s="16"/>
-      <c r="M3" s="16"/>
-      <c r="N3" s="16"/>
-      <c r="O3" s="16"/>
-      <c r="P3" s="16"/>
-    </row>
-    <row r="4" spans="1:19" s="9" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B4" s="60"/>
-      <c r="C4" s="66"/>
-      <c r="D4" s="61"/>
-      <c r="E4" s="61"/>
-      <c r="F4" s="61"/>
-      <c r="G4" s="61"/>
-      <c r="H4" s="61"/>
-      <c r="I4" s="61"/>
-      <c r="J4" s="67"/>
-      <c r="K4" s="16"/>
-      <c r="L4" s="16"/>
-      <c r="M4" s="16"/>
-      <c r="N4" s="16"/>
-      <c r="O4" s="16"/>
-      <c r="P4" s="16"/>
-    </row>
-    <row r="5" spans="1:19" s="9" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B5" s="62"/>
-      <c r="C5" s="63"/>
-      <c r="D5" s="63"/>
-      <c r="E5" s="63"/>
-      <c r="F5" s="63"/>
-      <c r="G5" s="63"/>
-      <c r="H5" s="63"/>
-      <c r="I5" s="63"/>
-      <c r="J5" s="68"/>
-      <c r="K5" s="16"/>
-      <c r="L5" s="16"/>
-      <c r="M5" s="16"/>
-      <c r="N5" s="16"/>
-      <c r="O5" s="16"/>
-      <c r="P5" s="16"/>
-    </row>
-    <row r="6" spans="1:19" s="9" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B6" s="62"/>
-      <c r="C6" s="63"/>
-      <c r="D6" s="63"/>
-      <c r="E6" s="63"/>
-      <c r="F6" s="63"/>
-      <c r="G6" s="63"/>
-      <c r="H6" s="63"/>
-      <c r="I6" s="63"/>
-      <c r="J6" s="68"/>
-      <c r="K6" s="16"/>
-      <c r="L6" s="16"/>
-      <c r="M6" s="16"/>
-      <c r="N6" s="16"/>
-      <c r="O6" s="16"/>
-      <c r="P6" s="16"/>
-    </row>
-    <row r="7" spans="1:19" s="9" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B7" s="64"/>
-      <c r="C7" s="65"/>
-      <c r="D7" s="65"/>
-      <c r="E7" s="65"/>
-      <c r="F7" s="65"/>
-      <c r="G7" s="65"/>
-      <c r="H7" s="65"/>
-      <c r="I7" s="65"/>
-      <c r="J7" s="69"/>
-      <c r="K7" s="16"/>
-      <c r="L7" s="16"/>
-      <c r="M7" s="16"/>
-      <c r="N7" s="16"/>
-      <c r="O7" s="16"/>
-      <c r="P7" s="16"/>
-    </row>
-    <row r="8" spans="1:19" s="9" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B8" s="19"/>
-      <c r="C8" s="19"/>
-      <c r="K8" s="16"/>
-      <c r="L8" s="16"/>
-      <c r="M8" s="16"/>
-      <c r="N8" s="16"/>
-      <c r="O8" s="16"/>
-      <c r="P8" s="16"/>
-    </row>
-    <row r="10" spans="1:19" ht="39" x14ac:dyDescent="0.35">
-      <c r="B10" s="11" t="s">
+      <c r="C1" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="D1" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="E1" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="E10" s="11" t="s">
+      <c r="F1" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="F10" s="11" t="s">
+      <c r="G1" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="G10" s="11" t="s">
+      <c r="H1" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="H10" s="11" t="s">
+      <c r="I1" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="I10" s="11" t="s">
+      <c r="J1" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="J10" s="11" t="s">
+      <c r="K1" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="L1" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="K10" s="11" t="s">
+      <c r="M1" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="L10" s="11" t="s">
+      <c r="N1" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="M10" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="N10" s="11" t="s">
+      <c r="O1" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="O10" s="11" t="s">
+      <c r="P1" s="55" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q1" s="57" t="s">
         <v>42</v>
       </c>
-      <c r="P10" s="55" t="s">
-        <v>18</v>
-      </c>
-      <c r="Q10" s="57" t="s">
+      <c r="R1" s="57" t="s">
         <v>43</v>
       </c>
-      <c r="R10" s="57" t="s">
+      <c r="S1" s="57" t="s">
         <v>44</v>
       </c>
-      <c r="S10" s="57" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="11" spans="1:19" s="12" customFormat="1" ht="105" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="20"/>
-      <c r="B11" s="13">
+    </row>
+    <row r="2" spans="1:19" s="12" customFormat="1" ht="105" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="20"/>
+      <c r="B2" s="13">
         <v>1</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="C2" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="D2" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="D11" s="14" t="s">
+      <c r="E2" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="E11" s="14" t="s">
+      <c r="F2" s="53">
+        <v>0</v>
+      </c>
+      <c r="G2" s="53">
+        <v>0</v>
+      </c>
+      <c r="H2" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="F11" s="53">
+      <c r="I2" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="J2" s="26"/>
+      <c r="K2" s="17"/>
+      <c r="L2" s="18"/>
+      <c r="M2" s="17"/>
+      <c r="N2" s="17"/>
+      <c r="O2" s="17"/>
+      <c r="P2" s="17"/>
+      <c r="Q2" s="56" t="s">
+        <v>56</v>
+      </c>
+      <c r="R2" s="58" t="s">
+        <v>46</v>
+      </c>
+      <c r="S2" s="58" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" s="12" customFormat="1" ht="105" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="20"/>
+      <c r="B3" s="13">
+        <v>2</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="D3" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="E3" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="F3" s="53">
         <v>0</v>
       </c>
-      <c r="G11" s="53">
+      <c r="G3" s="53">
         <v>0</v>
       </c>
-      <c r="H11" s="14" t="s">
+      <c r="H3" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="I3" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="I11" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="J11" s="26"/>
-      <c r="K11" s="17"/>
-      <c r="L11" s="18"/>
-      <c r="M11" s="17"/>
-      <c r="N11" s="17"/>
-      <c r="O11" s="17"/>
-      <c r="P11" s="17"/>
-      <c r="Q11" s="56" t="s">
-        <v>57</v>
-      </c>
-      <c r="R11" s="58" t="s">
-        <v>47</v>
-      </c>
-      <c r="S11" s="58" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="12" spans="1:19" s="12" customFormat="1" ht="105" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="20"/>
-      <c r="B12" s="13">
-        <v>2</v>
-      </c>
-      <c r="C12" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="D12" s="14" t="s">
-        <v>76</v>
-      </c>
-      <c r="E12" s="14" t="s">
-        <v>73</v>
-      </c>
-      <c r="F12" s="53">
-        <v>0</v>
-      </c>
-      <c r="G12" s="53">
-        <v>0</v>
-      </c>
-      <c r="H12" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="I12" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="J12" s="26"/>
-      <c r="K12" s="17"/>
-      <c r="L12" s="18"/>
-      <c r="M12" s="17"/>
-      <c r="N12" s="17"/>
-      <c r="O12" s="17"/>
-      <c r="P12" s="17"/>
-      <c r="Q12" s="56" t="s">
-        <v>57</v>
-      </c>
-      <c r="R12" s="58" t="s">
-        <v>47</v>
-      </c>
-      <c r="S12" s="58" t="s">
-        <v>47</v>
-      </c>
+      <c r="J3" s="26"/>
+      <c r="K3" s="17"/>
+      <c r="L3" s="18"/>
+      <c r="M3" s="17"/>
+      <c r="N3" s="17"/>
+      <c r="O3" s="17"/>
+      <c r="P3" s="17"/>
+      <c r="Q3" s="56" t="s">
+        <v>56</v>
+      </c>
+      <c r="R3" s="58" t="s">
+        <v>46</v>
+      </c>
+      <c r="S3" s="58" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="21"/>
+      <c r="H4" s="21"/>
+      <c r="I4" s="21"/>
+      <c r="K4" s="22"/>
+      <c r="L4" s="23"/>
+      <c r="M4" s="23"/>
+      <c r="N4" s="23"/>
+      <c r="O4" s="23"/>
+      <c r="P4" s="23"/>
+      <c r="Q4" s="25"/>
+    </row>
+    <row r="5" spans="1:19" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D5" s="21"/>
+      <c r="E5" s="21"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="21"/>
+      <c r="H5" s="21"/>
+      <c r="I5" s="21"/>
+      <c r="K5" s="22"/>
+      <c r="L5" s="23"/>
+      <c r="M5" s="23"/>
+      <c r="N5" s="23"/>
+      <c r="O5" s="23"/>
+      <c r="P5" s="23"/>
+      <c r="Q5" s="24"/>
+    </row>
+    <row r="6" spans="1:19" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D6" s="21"/>
+      <c r="E6" s="21"/>
+      <c r="F6" s="21"/>
+      <c r="G6" s="21"/>
+      <c r="H6" s="21"/>
+      <c r="I6" s="21"/>
+      <c r="K6" s="22"/>
+      <c r="L6" s="23"/>
+      <c r="M6" s="23"/>
+      <c r="N6" s="23"/>
+      <c r="O6" s="23"/>
+      <c r="P6" s="23"/>
+      <c r="Q6" s="24"/>
+    </row>
+    <row r="7" spans="1:19" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D7" s="21"/>
+      <c r="E7" s="21"/>
+      <c r="F7" s="21"/>
+      <c r="G7" s="21"/>
+      <c r="H7" s="21"/>
+      <c r="I7" s="21"/>
+      <c r="K7" s="22"/>
+      <c r="L7" s="23"/>
+      <c r="M7" s="23"/>
+      <c r="N7" s="23"/>
+      <c r="O7" s="23"/>
+      <c r="P7" s="23"/>
+      <c r="Q7" s="24"/>
+    </row>
+    <row r="8" spans="1:19" s="12" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D8" s="21"/>
+      <c r="E8" s="21"/>
+      <c r="F8" s="21"/>
+      <c r="G8" s="21"/>
+      <c r="H8" s="21"/>
+      <c r="I8" s="21"/>
+      <c r="K8" s="22"/>
+      <c r="L8" s="23"/>
+      <c r="M8" s="23"/>
+      <c r="N8" s="23"/>
+      <c r="O8" s="23"/>
+      <c r="P8" s="23"/>
+      <c r="Q8" s="24"/>
+    </row>
+    <row r="9" spans="1:19" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D9" s="21"/>
+      <c r="E9" s="21"/>
+      <c r="F9" s="21"/>
+      <c r="G9" s="21"/>
+      <c r="H9" s="21"/>
+      <c r="I9" s="21"/>
+      <c r="K9" s="22"/>
+      <c r="L9" s="23"/>
+      <c r="M9" s="23"/>
+      <c r="N9" s="23"/>
+      <c r="O9" s="23"/>
+      <c r="P9" s="23"/>
+      <c r="Q9" s="24"/>
+    </row>
+    <row r="10" spans="1:19" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="K10" s="23"/>
+      <c r="L10" s="23"/>
+      <c r="M10" s="23"/>
+      <c r="N10" s="23"/>
+      <c r="O10" s="23"/>
+      <c r="P10" s="23"/>
+      <c r="Q10" s="25"/>
+    </row>
+    <row r="11" spans="1:19" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="K11" s="23"/>
+      <c r="L11" s="23"/>
+      <c r="M11" s="23"/>
+      <c r="N11" s="23"/>
+      <c r="O11" s="23"/>
+      <c r="P11" s="23"/>
+      <c r="Q11" s="25"/>
+    </row>
+    <row r="12" spans="1:19" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="K12" s="23"/>
+      <c r="L12" s="23"/>
+      <c r="M12" s="23"/>
+      <c r="N12" s="23"/>
+      <c r="O12" s="23"/>
+      <c r="P12" s="23"/>
+      <c r="Q12" s="25"/>
     </row>
     <row r="13" spans="1:19" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="D13" s="21"/>
-      <c r="E13" s="21"/>
-      <c r="F13" s="21"/>
-      <c r="G13" s="21"/>
-      <c r="H13" s="21"/>
-      <c r="I13" s="21"/>
-      <c r="K13" s="22"/>
+      <c r="K13" s="23"/>
       <c r="L13" s="23"/>
       <c r="M13" s="23"/>
       <c r="N13" s="23"/>
@@ -2089,81 +2016,51 @@
       <c r="Q13" s="25"/>
     </row>
     <row r="14" spans="1:19" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="D14" s="21"/>
-      <c r="E14" s="21"/>
-      <c r="F14" s="21"/>
-      <c r="G14" s="21"/>
-      <c r="H14" s="21"/>
-      <c r="I14" s="21"/>
-      <c r="K14" s="22"/>
+      <c r="K14" s="23"/>
       <c r="L14" s="23"/>
       <c r="M14" s="23"/>
       <c r="N14" s="23"/>
       <c r="O14" s="23"/>
       <c r="P14" s="23"/>
-      <c r="Q14" s="24"/>
+      <c r="Q14" s="25"/>
     </row>
     <row r="15" spans="1:19" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="D15" s="21"/>
-      <c r="E15" s="21"/>
-      <c r="F15" s="21"/>
-      <c r="G15" s="21"/>
-      <c r="H15" s="21"/>
-      <c r="I15" s="21"/>
-      <c r="K15" s="22"/>
+      <c r="K15" s="23"/>
       <c r="L15" s="23"/>
       <c r="M15" s="23"/>
       <c r="N15" s="23"/>
       <c r="O15" s="23"/>
       <c r="P15" s="23"/>
-      <c r="Q15" s="24"/>
+      <c r="Q15" s="25"/>
     </row>
     <row r="16" spans="1:19" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="D16" s="21"/>
-      <c r="E16" s="21"/>
-      <c r="F16" s="21"/>
-      <c r="G16" s="21"/>
-      <c r="H16" s="21"/>
-      <c r="I16" s="21"/>
-      <c r="K16" s="22"/>
+      <c r="K16" s="23"/>
       <c r="L16" s="23"/>
       <c r="M16" s="23"/>
       <c r="N16" s="23"/>
       <c r="O16" s="23"/>
       <c r="P16" s="23"/>
-      <c r="Q16" s="24"/>
-    </row>
-    <row r="17" spans="4:17" s="12" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="D17" s="21"/>
-      <c r="E17" s="21"/>
-      <c r="F17" s="21"/>
-      <c r="G17" s="21"/>
-      <c r="H17" s="21"/>
-      <c r="I17" s="21"/>
-      <c r="K17" s="22"/>
+      <c r="Q16" s="25"/>
+    </row>
+    <row r="17" spans="11:17" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="K17" s="23"/>
       <c r="L17" s="23"/>
       <c r="M17" s="23"/>
       <c r="N17" s="23"/>
       <c r="O17" s="23"/>
       <c r="P17" s="23"/>
-      <c r="Q17" s="24"/>
-    </row>
-    <row r="18" spans="4:17" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="D18" s="21"/>
-      <c r="E18" s="21"/>
-      <c r="F18" s="21"/>
-      <c r="G18" s="21"/>
-      <c r="H18" s="21"/>
-      <c r="I18" s="21"/>
-      <c r="K18" s="22"/>
+      <c r="Q17" s="25"/>
+    </row>
+    <row r="18" spans="11:17" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="K18" s="23"/>
       <c r="L18" s="23"/>
       <c r="M18" s="23"/>
       <c r="N18" s="23"/>
       <c r="O18" s="23"/>
       <c r="P18" s="23"/>
-      <c r="Q18" s="24"/>
-    </row>
-    <row r="19" spans="4:17" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="Q18" s="25"/>
+    </row>
+    <row r="19" spans="11:17" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="K19" s="23"/>
       <c r="L19" s="23"/>
       <c r="M19" s="23"/>
@@ -2172,7 +2069,7 @@
       <c r="P19" s="23"/>
       <c r="Q19" s="25"/>
     </row>
-    <row r="20" spans="4:17" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="20" spans="11:17" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="K20" s="23"/>
       <c r="L20" s="23"/>
       <c r="M20" s="23"/>
@@ -2181,7 +2078,7 @@
       <c r="P20" s="23"/>
       <c r="Q20" s="25"/>
     </row>
-    <row r="21" spans="4:17" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="21" spans="11:17" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="K21" s="23"/>
       <c r="L21" s="23"/>
       <c r="M21" s="23"/>
@@ -2190,7 +2087,7 @@
       <c r="P21" s="23"/>
       <c r="Q21" s="25"/>
     </row>
-    <row r="22" spans="4:17" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="22" spans="11:17" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="K22" s="23"/>
       <c r="L22" s="23"/>
       <c r="M22" s="23"/>
@@ -2199,7 +2096,7 @@
       <c r="P22" s="23"/>
       <c r="Q22" s="25"/>
     </row>
-    <row r="23" spans="4:17" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="23" spans="11:17" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="K23" s="23"/>
       <c r="L23" s="23"/>
       <c r="M23" s="23"/>
@@ -2208,7 +2105,7 @@
       <c r="P23" s="23"/>
       <c r="Q23" s="25"/>
     </row>
-    <row r="24" spans="4:17" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="24" spans="11:17" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="K24" s="23"/>
       <c r="L24" s="23"/>
       <c r="M24" s="23"/>
@@ -2217,7 +2114,7 @@
       <c r="P24" s="23"/>
       <c r="Q24" s="25"/>
     </row>
-    <row r="25" spans="4:17" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="25" spans="11:17" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="K25" s="23"/>
       <c r="L25" s="23"/>
       <c r="M25" s="23"/>
@@ -2226,7 +2123,7 @@
       <c r="P25" s="23"/>
       <c r="Q25" s="25"/>
     </row>
-    <row r="26" spans="4:17" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="26" spans="11:17" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="K26" s="23"/>
       <c r="L26" s="23"/>
       <c r="M26" s="23"/>
@@ -2235,7 +2132,7 @@
       <c r="P26" s="23"/>
       <c r="Q26" s="25"/>
     </row>
-    <row r="27" spans="4:17" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="27" spans="11:17" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="K27" s="23"/>
       <c r="L27" s="23"/>
       <c r="M27" s="23"/>
@@ -2244,92 +2141,8 @@
       <c r="P27" s="23"/>
       <c r="Q27" s="25"/>
     </row>
-    <row r="28" spans="4:17" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="K28" s="23"/>
-      <c r="L28" s="23"/>
-      <c r="M28" s="23"/>
-      <c r="N28" s="23"/>
-      <c r="O28" s="23"/>
-      <c r="P28" s="23"/>
-      <c r="Q28" s="25"/>
-    </row>
-    <row r="29" spans="4:17" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="K29" s="23"/>
-      <c r="L29" s="23"/>
-      <c r="M29" s="23"/>
-      <c r="N29" s="23"/>
-      <c r="O29" s="23"/>
-      <c r="P29" s="23"/>
-      <c r="Q29" s="25"/>
-    </row>
-    <row r="30" spans="4:17" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="K30" s="23"/>
-      <c r="L30" s="23"/>
-      <c r="M30" s="23"/>
-      <c r="N30" s="23"/>
-      <c r="O30" s="23"/>
-      <c r="P30" s="23"/>
-      <c r="Q30" s="25"/>
-    </row>
-    <row r="31" spans="4:17" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="K31" s="23"/>
-      <c r="L31" s="23"/>
-      <c r="M31" s="23"/>
-      <c r="N31" s="23"/>
-      <c r="O31" s="23"/>
-      <c r="P31" s="23"/>
-      <c r="Q31" s="25"/>
-    </row>
-    <row r="32" spans="4:17" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="K32" s="23"/>
-      <c r="L32" s="23"/>
-      <c r="M32" s="23"/>
-      <c r="N32" s="23"/>
-      <c r="O32" s="23"/>
-      <c r="P32" s="23"/>
-      <c r="Q32" s="25"/>
-    </row>
-    <row r="33" spans="11:17" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="K33" s="23"/>
-      <c r="L33" s="23"/>
-      <c r="M33" s="23"/>
-      <c r="N33" s="23"/>
-      <c r="O33" s="23"/>
-      <c r="P33" s="23"/>
-      <c r="Q33" s="25"/>
-    </row>
-    <row r="34" spans="11:17" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="K34" s="23"/>
-      <c r="L34" s="23"/>
-      <c r="M34" s="23"/>
-      <c r="N34" s="23"/>
-      <c r="O34" s="23"/>
-      <c r="P34" s="23"/>
-      <c r="Q34" s="25"/>
-    </row>
-    <row r="35" spans="11:17" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="K35" s="23"/>
-      <c r="L35" s="23"/>
-      <c r="M35" s="23"/>
-      <c r="N35" s="23"/>
-      <c r="O35" s="23"/>
-      <c r="P35" s="23"/>
-      <c r="Q35" s="25"/>
-    </row>
-    <row r="36" spans="11:17" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="K36" s="23"/>
-      <c r="L36" s="23"/>
-      <c r="M36" s="23"/>
-      <c r="N36" s="23"/>
-      <c r="O36" s="23"/>
-      <c r="P36" s="23"/>
-      <c r="Q36" s="25"/>
-    </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B4:J7"/>
-  </mergeCells>
-  <conditionalFormatting sqref="Q11 Q13:Q36">
+  <conditionalFormatting sqref="Q2 Q4:Q27">
     <cfRule type="cellIs" dxfId="5" priority="7" operator="equal">
       <formula>"Green"</formula>
     </cfRule>
@@ -2340,7 +2153,7 @@
       <formula>"Red"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q12">
+  <conditionalFormatting sqref="Q3">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"Green"</formula>
     </cfRule>
@@ -2352,7 +2165,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q11:Q36" xr:uid="{4E9472C3-0F59-436D-B36A-0DE15C8EE443}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q2:Q27" xr:uid="{4E9472C3-0F59-436D-B36A-0DE15C8EE443}">
       <formula1>"Red, Amber, Green"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2361,7 +2174,6 @@
   <headerFooter>
     <oddFooter>&amp;C&amp;1#&amp;"Calibri"&amp;10&amp;K000000OFFICIAL-SENSITIVE</oddFooter>
   </headerFooter>
-  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -2389,58 +2201,58 @@
     </row>
     <row r="2" spans="1:8" ht="138.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3"/>
-      <c r="B2" s="70" t="s">
+      <c r="B2" s="66" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="C2" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="D2" s="4" t="s">
+      <c r="F2" s="69" t="s">
         <v>50</v>
       </c>
-      <c r="F2" s="73" t="s">
+      <c r="G2" s="54" t="s">
+        <v>47</v>
+      </c>
+      <c r="H2" s="54" t="s">
         <v>51</v>
-      </c>
-      <c r="G2" s="54" t="s">
-        <v>48</v>
-      </c>
-      <c r="H2" s="54" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="144.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3"/>
-      <c r="B3" s="71"/>
+      <c r="B3" s="67"/>
       <c r="C3" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="E3" s="5"/>
+      <c r="F3" s="69"/>
+      <c r="G3" s="54" t="s">
         <v>54</v>
       </c>
-      <c r="E3" s="5"/>
-      <c r="F3" s="73"/>
-      <c r="G3" s="54" t="s">
+      <c r="H3" s="54" t="s">
         <v>55</v>
-      </c>
-      <c r="H3" s="54" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="121.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="3"/>
-      <c r="B4" s="72"/>
+      <c r="B4" s="68"/>
       <c r="C4" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="F4" s="69"/>
+      <c r="G4" s="54" t="s">
+        <v>46</v>
+      </c>
+      <c r="H4" s="54" t="s">
         <v>58</v>
-      </c>
-      <c r="F4" s="73"/>
-      <c r="G4" s="54" t="s">
-        <v>47</v>
-      </c>
-      <c r="H4" s="54" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
@@ -2489,22 +2301,22 @@
   <sheetData>
     <row r="2" spans="2:10" ht="29" x14ac:dyDescent="0.35">
       <c r="B2" s="28" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" spans="2:10" ht="49" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B4" s="28" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B5" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.35">
       <c r="D6" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="7" spans="2:10" ht="23.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -2513,7 +2325,7 @@
       <c r="F7" s="38"/>
       <c r="G7" s="38"/>
       <c r="H7" s="39" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I7" s="38"/>
       <c r="J7" s="35"/>
@@ -2525,63 +2337,63 @@
     <row r="9" spans="2:10" x14ac:dyDescent="0.35">
       <c r="D9" s="41"/>
       <c r="G9" s="32" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H9" s="32" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I9" s="32" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J9" s="29"/>
     </row>
     <row r="10" spans="2:10" x14ac:dyDescent="0.35">
       <c r="D10" s="41"/>
       <c r="F10" s="31" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G10" s="36" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="H10" s="36" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="I10" s="36" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J10" s="29"/>
     </row>
     <row r="11" spans="2:10" x14ac:dyDescent="0.35">
       <c r="D11" s="42" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F11" s="31" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G11" s="36" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="H11" s="36" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I11" s="36" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="J11" s="29"/>
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.35">
       <c r="D12" s="41"/>
       <c r="F12" s="31" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G12" s="36" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H12" s="36" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="I12" s="36" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="J12" s="29"/>
     </row>
@@ -2596,12 +2408,12 @@
     </row>
     <row r="15" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B15" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="16" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B16" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -2619,17 +2431,17 @@
   <sheetData>
     <row r="2" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B3" s="59" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>